<commit_message>
Update Term 3 timetable and add senior dashboards
</commit_message>
<xml_diff>
--- a/drumming_timetable.xlsx
+++ b/drumming_timetable.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Term 3 Timetable" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,36 +413,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>9:40</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
         <is>
           <t>11:05</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>11:35</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>12:45</t>
         </is>
@@ -488,6 +496,16 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>Chance</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Huarya</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>Harvey</t>
         </is>
       </c>
@@ -500,7 +518,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Huarya</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -519,6 +537,16 @@
         </is>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Chance</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>
@@ -532,12 +560,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Herschell</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Huarya</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -551,6 +579,16 @@
         </is>
       </c>
       <c r="F4" t="inlineStr">
+        <is>
+          <t>Herschell</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>
@@ -564,17 +602,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bailey</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Herschell</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Huarya</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -583,6 +621,16 @@
         </is>
       </c>
       <c r="F5" t="inlineStr">
+        <is>
+          <t>Bailey</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Herschell</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>
@@ -596,25 +644,35 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Herschell</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Bailey</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Herschell</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Huarya</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
+        <is>
+          <t>Luke</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Bailey</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>
@@ -628,25 +686,35 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Bailey</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Herschell</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Bailey</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Herschell</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
+        <is>
+          <t>Huarya</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Luke</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>
@@ -660,25 +728,35 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Herschell</t>
+          <t>Luke</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Bailey</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Herschell</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Bailey</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
+        <is>
+          <t>Chance</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Huarya</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>
@@ -692,25 +770,35 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bailey</t>
+          <t>Huarya</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Herschell</t>
+          <t>Luke</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Bailey</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Herschell</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Chance</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>
@@ -724,25 +812,35 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Bailey</t>
+          <t>Huarya</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Herschell</t>
+          <t>Luke</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Bailey</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
+        <is>
+          <t>Herschell</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>
@@ -761,20 +859,30 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Bailey</t>
+          <t>Huarya</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Herschell</t>
+          <t>Luke</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
+        <is>
+          <t>Bailey</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Herschell</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>

</xml_diff>

<commit_message>
Update Term 3 timetable and add senior dashboards (#2)
Co-authored-by: copilot-swe-agent[bot] <198982749+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/drumming_timetable.xlsx
+++ b/drumming_timetable.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Term 3 Timetable" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,36 +413,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>9:40</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
         <is>
           <t>11:05</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>11:35</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>12:45</t>
         </is>
@@ -488,6 +496,16 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>Chance</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Huarya</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>Harvey</t>
         </is>
       </c>
@@ -500,7 +518,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Huarya</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -519,6 +537,16 @@
         </is>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Chance</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>
@@ -532,12 +560,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Herschell</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Huarya</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -551,6 +579,16 @@
         </is>
       </c>
       <c r="F4" t="inlineStr">
+        <is>
+          <t>Herschell</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>
@@ -564,17 +602,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bailey</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Herschell</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Huarya</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -583,6 +621,16 @@
         </is>
       </c>
       <c r="F5" t="inlineStr">
+        <is>
+          <t>Bailey</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Herschell</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>
@@ -596,25 +644,35 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Herschell</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Bailey</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Herschell</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Huarya</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
+        <is>
+          <t>Luke</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Bailey</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>
@@ -628,25 +686,35 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Bailey</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Herschell</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Bailey</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Herschell</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
+        <is>
+          <t>Huarya</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Luke</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>
@@ -660,25 +728,35 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Herschell</t>
+          <t>Luke</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Bailey</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Herschell</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Bailey</t>
+          <t>Thomas</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
+        <is>
+          <t>Chance</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Huarya</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>
@@ -692,25 +770,35 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bailey</t>
+          <t>Huarya</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Herschell</t>
+          <t>Luke</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Bailey</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Herschell</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Chance</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>
@@ -724,25 +812,35 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Bailey</t>
+          <t>Huarya</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Herschell</t>
+          <t>Luke</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Bailey</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
+        <is>
+          <t>Herschell</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>
@@ -761,20 +859,30 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Luke</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Bailey</t>
+          <t>Huarya</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Herschell</t>
+          <t>Luke</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
+        <is>
+          <t>Bailey</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Herschell</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>Harvey</t>
         </is>

</xml_diff>